<commit_message>
Populate XLSX from json_output
</commit_message>
<xml_diff>
--- a/260305_DB-Strcuture_05.xlsx
+++ b/260305_DB-Strcuture_05.xlsx
@@ -5667,7 +5667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M104"/>
+  <dimension ref="A1:B104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.42578125" customWidth="1" min="1" max="1"/>
@@ -16179,7 +16179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1146"/>
+  <dimension ref="A1:C1146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.42578125" customWidth="1" min="1" max="1"/>

</xml_diff>